<commit_message>
Created initial Power BI file
</commit_message>
<xml_diff>
--- a/Data/Cleaned/Aster Retail Holdings Pivot.xlsx
+++ b/Data/Cleaned/Aster Retail Holdings Pivot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\Infotact-Solution-Project-1\Data\Cleaned\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AD446D4-3908-4599-B1BD-1B2B77EBDD96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D32B3AC-D13F-43FB-A5EC-E124A87EF1AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33854,6 +33854,7 @@
   <cols>
     <col min="1" max="1" width="16.33203125" customWidth="1"/>
     <col min="2" max="2" width="12.109375" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" customWidth="1"/>
     <col min="5" max="5" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.109375" bestFit="1" customWidth="1"/>
@@ -34251,143 +34252,143 @@
     <mergeCell ref="N2:R2"/>
   </mergeCells>
   <conditionalFormatting pivot="1" sqref="J4 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15">
-    <cfRule type="cellIs" dxfId="58" priority="32" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="32" operator="greaterThan">
       <formula>60000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="J4 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15">
-    <cfRule type="cellIs" dxfId="57" priority="31" operator="lessThan">
+    <cfRule type="cellIs" dxfId="30" priority="31" operator="lessThan">
       <formula>60000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="J4 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15">
-    <cfRule type="cellIs" dxfId="56" priority="30" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="30" operator="greaterThan">
       <formula>90000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K19">
-    <cfRule type="cellIs" dxfId="55" priority="29" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="28" priority="29" operator="greaterThan">
       <formula>60000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K19">
-    <cfRule type="cellIs" dxfId="54" priority="28" operator="lessThan">
+    <cfRule type="cellIs" dxfId="27" priority="28" operator="lessThan">
       <formula>60000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K19">
-    <cfRule type="cellIs" dxfId="53" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="27" operator="greaterThan">
       <formula>90000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="O5:Q10">
-    <cfRule type="cellIs" dxfId="52" priority="26" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="25" priority="26" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="O5:Q10">
-    <cfRule type="cellIs" dxfId="51" priority="25" operator="between">
+    <cfRule type="cellIs" dxfId="24" priority="25" operator="between">
       <formula>30000</formula>
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="O5:Q10">
-    <cfRule type="cellIs" dxfId="50" priority="24" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="24" operator="lessThan">
       <formula>30000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="O5:Q10">
-    <cfRule type="cellIs" dxfId="49" priority="23" operator="between">
+    <cfRule type="cellIs" dxfId="22" priority="23" operator="between">
       <formula>30000</formula>
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="O5:Q10">
-    <cfRule type="cellIs" dxfId="48" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
       <formula>30000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="O5:Q10">
-    <cfRule type="cellIs" dxfId="47" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="21" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="O5:Q10">
-    <cfRule type="cellIs" dxfId="46" priority="20" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="19" priority="20" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R19">
-    <cfRule type="cellIs" dxfId="45" priority="19" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="19" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R19">
-    <cfRule type="cellIs" dxfId="44" priority="18" operator="between">
+    <cfRule type="cellIs" dxfId="17" priority="18" operator="between">
       <formula>30000</formula>
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R19">
-    <cfRule type="cellIs" dxfId="43" priority="17" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="17" operator="lessThan">
       <formula>30000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R19">
-    <cfRule type="cellIs" dxfId="42" priority="16" operator="between">
+    <cfRule type="cellIs" dxfId="15" priority="16" operator="between">
       <formula>30000</formula>
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R19">
-    <cfRule type="cellIs" dxfId="41" priority="15" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="15" operator="lessThan">
       <formula>30000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R19">
-    <cfRule type="cellIs" dxfId="40" priority="14" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R19">
-    <cfRule type="cellIs" dxfId="39" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="13" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R20">
-    <cfRule type="cellIs" dxfId="38" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R20">
-    <cfRule type="cellIs" dxfId="37" priority="11" operator="between">
+    <cfRule type="cellIs" dxfId="10" priority="11" operator="between">
       <formula>30000</formula>
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R20">
-    <cfRule type="cellIs" dxfId="36" priority="10" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="10" operator="lessThan">
       <formula>30000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R20">
-    <cfRule type="cellIs" dxfId="35" priority="9" operator="between">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="between">
       <formula>30000</formula>
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R20">
-    <cfRule type="cellIs" dxfId="34" priority="8" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="lessThan">
       <formula>30000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R20">
-    <cfRule type="cellIs" dxfId="33" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R20">
-    <cfRule type="cellIs" dxfId="32" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
       <formula>40655</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>